<commit_message>
retailer: publish imported establishments to shared maps and list owned locations
</commit_message>
<xml_diff>
--- a/yokup-site/templates/ubicaciones-retailer.xlsx
+++ b/yokup-site/templates/ubicaciones-retailer.xlsx
@@ -445,7 +445,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -547,15 +547,23 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Admira</v>
+        <v>Mapas públicos</v>
       </c>
       <c r="B14" t="str">
-        <v>Las altas quedan pendientes hasta que el servicio central confirma su registro.</v>
+        <v>Al confirmar se publican nombre, tipo, dirección y coordenadas en admira.app y clearchannel.tv.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Equipos</v>
+      </c>
+      <c r="B15" t="str">
+        <v>La importación no crea pantallas ni activa su monitorización.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>